<commit_message>
Added line chart visualization to analysis.xlsx
</commit_message>
<xml_diff>
--- a/result_analysis/analysis.xlsx
+++ b/result_analysis/analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tintin/Desktop/Projects/credit_risk_model/result_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8831DDB9-1849-5340-962D-71CBF2B20E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B792EA5-9AF6-E945-B565-DA255D487101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="800" windowWidth="28040" windowHeight="17440" activeTab="3" xr2:uid="{61FC1A9A-6CB0-D841-9DA7-4D6ECF9C438C}"/>
   </bookViews>
@@ -269,21 +269,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill>
@@ -390,6 +376,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFC90F19"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -399,6 +390,1531 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Maximize</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Profit against Predicted Probability of Default</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Total Profit</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="22225" cap="rnd" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="accent2"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="20000"/>
+                    <a:lumOff val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:ln>
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="accent6">
+                          <a:lumMod val="75000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="6"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="8"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="9"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:spAutoFit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:srgbClr val="FF0000"/>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="t"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-079E-F44A-B5E1-B670670C29C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="dk1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>pivot_table!$D$4:$D$13</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0.17496599286467901</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.35881366224141897</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.47584258697556497</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.56482777819684904</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.63757566072097405</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.68823276453429405</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.73607145012303798</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.790000147675743</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.84607193303260098</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.88753490911426602</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>pivot_table!$L$4:$L$13</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>3400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12400</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-3800</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-29800</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-60000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-88800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-116200</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-146400</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-173800</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-201200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-079E-F44A-B5E1-B670670C29C0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="t"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:dropLines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="35000"/>
+                  <a:lumOff val="65000"/>
+                  <a:alpha val="33000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:dropLines>
+        <c:smooth val="0"/>
+        <c:axId val="907705135"/>
+        <c:axId val="907707743"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="907705135"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Model Predicted Probability of Default</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.37937524573177817"/>
+              <c:y val="0.90743766329059639"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="dk1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="907707743"/>
+        <c:crossesAt val="-250000"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="907707743"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="907705135"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="100000">
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="0">
+              <a:schemeClr val="lt1"/>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="lt1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="230">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" b="0" kern="1200" spc="20" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="2">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="1"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:shade val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="2">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="1"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:shade val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="22225" cap="rnd" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="4"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+            <a:alpha val="33000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill>
+        <a:gsLst>
+          <a:gs pos="100000">
+            <a:schemeClr val="lt1">
+              <a:lumMod val="95000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="0">
+            <a:schemeClr val="lt1"/>
+          </a:gs>
+        </a:gsLst>
+        <a:lin ang="5400000" scaled="0"/>
+      </a:gradFill>
+    </cs:spPr>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" kern="1200" cap="none" spc="20" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" spc="20" baseline="0"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1174814</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>42269</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>538480</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>142713</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04606F60-F557-0424-0946-48AA077DEE4E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4137,7 +5653,7 @@
     <dataField name="Min of Probability_Default" fld="3" subtotal="min" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="3">
+    <format dxfId="1">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -4149,7 +5665,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="0">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -4179,7 +5695,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00A61614-C026-F049-8D7D-B2C5D987FC7D}" name="Table1" displayName="Table1" ref="A1:G401" totalsRowShown="0" headerRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00A61614-C026-F049-8D7D-B2C5D987FC7D}" name="Table1" displayName="Table1" ref="A1:G401" totalsRowShown="0" headerRowDxfId="10">
   <autoFilter ref="A1:G401" xr:uid="{00A61614-C026-F049-8D7D-B2C5D987FC7D}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E401">
     <sortCondition descending="1" ref="D1:D401"/>
@@ -4187,13 +5703,13 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{A33D2E8F-C4FE-744C-B6EA-6D08D082939C}" name="index"/>
     <tableColumn id="2" xr3:uid="{B6ED8025-A452-0545-83F5-078527E9E23D}" name="Actual Outcome"/>
-    <tableColumn id="3" xr3:uid="{482B43F2-766E-4344-A44D-179FE0BFAA6E}" name="Probability_Safe" dataDxfId="11" dataCellStyle="Percent"/>
-    <tableColumn id="4" xr3:uid="{797E6CBE-CC91-DD44-BA30-CDAD50AEEDE6}" name="Probability_Default" dataDxfId="10" dataCellStyle="Percent"/>
+    <tableColumn id="3" xr3:uid="{482B43F2-766E-4344-A44D-179FE0BFAA6E}" name="Probability_Safe" dataDxfId="9" dataCellStyle="Percent"/>
+    <tableColumn id="4" xr3:uid="{797E6CBE-CC91-DD44-BA30-CDAD50AEEDE6}" name="Probability_Default" dataDxfId="8" dataCellStyle="Percent"/>
     <tableColumn id="5" xr3:uid="{8F649A08-FC6F-404F-ADA2-2B66671FF421}" name="Predicted Outcome"/>
-    <tableColumn id="8" xr3:uid="{B81D5698-9F0B-9B45-A8E1-F4463C47F39B}" name="True Positive" dataDxfId="7">
+    <tableColumn id="8" xr3:uid="{B81D5698-9F0B-9B45-A8E1-F4463C47F39B}" name="True Positive" dataDxfId="5">
       <calculatedColumnFormula>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{47E82062-EA15-D14E-9771-A0661A0DD882}" name="Decile" dataDxfId="8">
+    <tableColumn id="7" xr3:uid="{47E82062-EA15-D14E-9771-A0661A0DD882}" name="Decile" dataDxfId="6">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(MAX(IF(Table2[Probability_Default]&lt;Table1[[#This Row],[Probability_Default]],Table2[Probability_Default])),Table2[Probability_Default],Table2[Decile],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4206,7 +5722,7 @@
   <autoFilter ref="J1:K10" xr:uid="{67FE4D2D-295A-FD43-B1A1-4828D3A56142}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{85908CF2-458E-DC4E-9C8D-DD7ACB04BE26}" name="Decile"/>
-    <tableColumn id="2" xr3:uid="{829CD0D6-0304-6044-B4C2-6E080E4914FE}" name="Probability_Default" dataDxfId="9" dataCellStyle="Percent"/>
+    <tableColumn id="2" xr3:uid="{829CD0D6-0304-6044-B4C2-6E080E4914FE}" name="Probability_Default" dataDxfId="7" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4237,16 +5753,16 @@
     <tableColumn id="3" xr3:uid="{4DF9A59C-7522-3B4F-9E93-B8FD4567A10D}" name="Cumulative Defaults">
       <calculatedColumnFormula>SUM($C$4:C4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0B23C047-C32D-3A4B-BD60-B8C615AA7BB4}" name="Cumulative % of Defaults" dataDxfId="6" dataCellStyle="Percent">
+    <tableColumn id="5" xr3:uid="{0B23C047-C32D-3A4B-BD60-B8C615AA7BB4}" name="Cumulative % of Defaults" dataDxfId="4" dataCellStyle="Percent">
       <calculatedColumnFormula>(H4)/$H$13</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{F7D20E3F-556C-1940-82F2-43B673E2D5D4}" name="Cumulative Safe Loans">
       <calculatedColumnFormula>SUM($G$4:G4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{828E05FA-42DB-2D44-82BC-3CE97F0BCB66}" name="Cumulative % of Safe Loans" dataDxfId="5" dataCellStyle="Percent">
+    <tableColumn id="6" xr3:uid="{828E05FA-42DB-2D44-82BC-3CE97F0BCB66}" name="Cumulative % of Safe Loans" dataDxfId="3" dataCellStyle="Percent">
       <calculatedColumnFormula>(J4)/$J$13</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B38B3630-1B13-C646-85B9-356D48FF1C8B}" name="Total Profit" dataDxfId="4" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{B38B3630-1B13-C646-85B9-356D48FF1C8B}" name="Total Profit" dataDxfId="2" dataCellStyle="Percent">
       <calculatedColumnFormula>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -23245,8 +24761,9 @@
     <mergeCell ref="G18:H18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>